<commit_message>
Updated results somewhat, figures, tables
</commit_message>
<xml_diff>
--- a/Results/mainresults.xlsx
+++ b/Results/mainresults.xlsx
@@ -418,22 +418,22 @@
         </is>
       </c>
       <c r="D2">
-        <v>0.01708025645379275</v>
+        <v>0.01987143426751635</v>
       </c>
       <c r="E2">
-        <v>0.004843345661506257</v>
+        <v>0.004961787724162165</v>
       </c>
       <c r="F2">
-        <v>3.526540876390985</v>
+        <v>4.004894076937117</v>
       </c>
       <c r="G2">
-        <v>0.0004210261680469568</v>
+        <v>6.204527671571261E-05</v>
       </c>
       <c r="H2">
-        <v>0.007587473392562164</v>
+        <v>0.01014650902922555</v>
       </c>
       <c r="I2">
-        <v>0.02657303951502333</v>
+        <v>0.02959635950580716</v>
       </c>
     </row>
     <row r="3">
@@ -453,22 +453,22 @@
         </is>
       </c>
       <c r="D3">
-        <v>0.003005974907376937</v>
+        <v>0.0001832961695471341</v>
       </c>
       <c r="E3">
-        <v>0.007040280311046222</v>
+        <v>0.007262161922928861</v>
       </c>
       <c r="F3">
-        <v>0.4269680715213218</v>
+        <v>0.02523989019969552</v>
       </c>
       <c r="G3">
-        <v>0.6694025833718116</v>
+        <v>0.9798636193031247</v>
       </c>
       <c r="H3">
-        <v>-0.0107927209433401</v>
+        <v>-0.01405027964929157</v>
       </c>
       <c r="I3">
-        <v>0.01680467075809398</v>
+        <v>0.01441687198838584</v>
       </c>
     </row>
     <row r="4">
@@ -488,22 +488,22 @@
         </is>
       </c>
       <c r="D4">
-        <v>0.01366720831589043</v>
+        <v>0.01798467081903042</v>
       </c>
       <c r="E4">
-        <v>0.006830674707355186</v>
+        <v>0.0071138277807318</v>
       </c>
       <c r="F4">
-        <v>2.000857733888828</v>
+        <v>2.528128508781574</v>
       </c>
       <c r="G4">
-        <v>0.0454077235420647</v>
+        <v>0.01146723701557349</v>
       </c>
       <c r="H4">
-        <v>0.0002793318993655949</v>
+        <v>0.004041824576575596</v>
       </c>
       <c r="I4">
-        <v>0.02705508473241527</v>
+        <v>0.03192751706148525</v>
       </c>
     </row>
     <row r="5">
@@ -523,22 +523,22 @@
         </is>
       </c>
       <c r="D5">
-        <v>0.02240712440317428</v>
+        <v>0.002720766972376285</v>
       </c>
       <c r="E5">
-        <v>0.008532703049966143</v>
+        <v>0.008423904286238954</v>
       </c>
       <c r="F5">
-        <v>2.626028852986181</v>
+        <v>0.3229817053858092</v>
       </c>
       <c r="G5">
-        <v>0.00863874943058061</v>
+        <v>0.746709097169707</v>
       </c>
       <c r="H5">
-        <v>0.00568333373446557</v>
+        <v>-0.01378978203786465</v>
       </c>
       <c r="I5">
-        <v>0.03913091507188299</v>
+        <v>0.01923131598261722</v>
       </c>
     </row>
     <row r="6">
@@ -558,22 +558,22 @@
         </is>
       </c>
       <c r="D6">
-        <v>0.01168525150008886</v>
+        <v>0.01623324829873208</v>
       </c>
       <c r="E6">
-        <v>0.007692868461147037</v>
+        <v>0.007447953647820331</v>
       </c>
       <c r="F6">
-        <v>1.518971962032813</v>
+        <v>2.179558180183196</v>
       </c>
       <c r="G6">
-        <v>0.1287695536044858</v>
+        <v>0.02929022758439538</v>
       </c>
       <c r="H6">
-        <v>-0.003392493621563394</v>
+        <v>0.001635527390480515</v>
       </c>
       <c r="I6">
-        <v>0.02676299662174112</v>
+        <v>0.03083096920698365</v>
       </c>
     </row>
     <row r="7">
@@ -593,22 +593,22 @@
         </is>
       </c>
       <c r="D7">
-        <v>0.01602285347315182</v>
+        <v>0.01333478743963215</v>
       </c>
       <c r="E7">
-        <v>0.01764110780246534</v>
+        <v>0.01790489929032319</v>
       </c>
       <c r="F7">
-        <v>0.9082679870542276</v>
+        <v>0.7447563498354336</v>
       </c>
       <c r="G7">
-        <v>0.3637366517467547</v>
+        <v>0.4564190271047672</v>
       </c>
       <c r="H7">
-        <v>-0.01855308246706877</v>
+        <v>-0.02175817031621808</v>
       </c>
       <c r="I7">
-        <v>0.05059878941337241</v>
+        <v>0.04842774519548237</v>
       </c>
     </row>
     <row r="8">
@@ -628,22 +628,22 @@
         </is>
       </c>
       <c r="D8">
-        <v>0.03039774046696423</v>
+        <v>0.02364277775111993</v>
       </c>
       <c r="E8">
-        <v>0.01472018884724969</v>
+        <v>0.01501968953997905</v>
       </c>
       <c r="F8">
-        <v>2.06503739744098</v>
+        <v>1.5741189382236</v>
       </c>
       <c r="G8">
-        <v>0.03891946194680391</v>
+        <v>0.1154599550681725</v>
       </c>
       <c r="H8">
-        <v>0.001546700480726675</v>
+        <v>-0.005795272806211973</v>
       </c>
       <c r="I8">
-        <v>0.05924878045320178</v>
+        <v>0.05308082830845184</v>
       </c>
     </row>
     <row r="9">
@@ -663,22 +663,22 @@
         </is>
       </c>
       <c r="D9">
-        <v>-0.004920971826940894</v>
+        <v>-0.006886807422543868</v>
       </c>
       <c r="E9">
-        <v>0.01740002022209906</v>
+        <v>0.01799047069112808</v>
       </c>
       <c r="F9">
-        <v>-0.2828141441290376</v>
+        <v>-0.3828030706244981</v>
       </c>
       <c r="G9">
-        <v>0.77731931134486</v>
+        <v>0.7018657845763321</v>
       </c>
       <c r="H9">
-        <v>-0.03902438479252368</v>
+        <v>-0.04214748204207832</v>
       </c>
       <c r="I9">
-        <v>0.02918244113864189</v>
+        <v>0.02837386719699058</v>
       </c>
     </row>
     <row r="10">
@@ -698,22 +698,22 @@
         </is>
       </c>
       <c r="D10">
-        <v>-0.02232310169965371</v>
+        <v>-0.01956303578930273</v>
       </c>
       <c r="E10">
-        <v>0.01696438900535614</v>
+        <v>0.01788427029661514</v>
       </c>
       <c r="F10">
-        <v>-1.315880088142619</v>
+        <v>-1.09386826886671</v>
       </c>
       <c r="G10">
-        <v>0.1882142929306335</v>
+        <v>0.2740127572276837</v>
       </c>
       <c r="H10">
-        <v>-0.05557269316987901</v>
+        <v>-0.05461556146044787</v>
       </c>
       <c r="I10">
-        <v>0.01092648977057158</v>
+        <v>0.0154894898818424</v>
       </c>
     </row>
     <row r="11">
@@ -733,22 +733,22 @@
         </is>
       </c>
       <c r="D11">
-        <v>0.05141870792023887</v>
+        <v>0.04947352423294215</v>
       </c>
       <c r="E11">
-        <v>0.00643749962424067</v>
+        <v>0.006645543852715086</v>
       </c>
       <c r="F11">
-        <v>7.987372570340759</v>
+        <v>7.44461632176716</v>
       </c>
       <c r="G11">
-        <v>1.378450217515444E-15</v>
+        <v>9.722657216075414E-14</v>
       </c>
       <c r="H11">
-        <v>0.03880144050623703</v>
+        <v>0.03644849762393903</v>
       </c>
       <c r="I11">
-        <v>0.06403597533424071</v>
+        <v>0.06249855084194527</v>
       </c>
     </row>
     <row r="12">
@@ -768,22 +768,22 @@
         </is>
       </c>
       <c r="D12">
-        <v>0.04829335352731845</v>
+        <v>0.04586855848303279</v>
       </c>
       <c r="E12">
-        <v>0.009654282901214225</v>
+        <v>0.009834807506769197</v>
       </c>
       <c r="F12">
-        <v>5.002272465129913</v>
+        <v>4.66389997480499</v>
       </c>
       <c r="G12">
-        <v>5.66584355859359E-07</v>
+        <v>3.102722380556536E-06</v>
       </c>
       <c r="H12">
-        <v>0.02937130674437771</v>
+        <v>0.026592689974881</v>
       </c>
       <c r="I12">
-        <v>0.06721540031025919</v>
+        <v>0.06514442699118458</v>
       </c>
     </row>
     <row r="13">
@@ -803,22 +803,22 @@
         </is>
       </c>
       <c r="D13">
-        <v>0.0492175921003625</v>
+        <v>0.06126268708049752</v>
       </c>
       <c r="E13">
-        <v>0.008643507747685927</v>
+        <v>0.009033438663248823</v>
       </c>
       <c r="F13">
-        <v>5.694168795479963</v>
+        <v>6.78176820192907</v>
       </c>
       <c r="G13">
-        <v>1.239743896090638E-08</v>
+        <v>1.187138407869338E-11</v>
       </c>
       <c r="H13">
-        <v>0.03227662821480517</v>
+        <v>0.04355747264397818</v>
       </c>
       <c r="I13">
-        <v>0.06615855598591983</v>
+        <v>0.07896790151701685</v>
       </c>
     </row>
     <row r="14">
@@ -838,22 +838,22 @@
         </is>
       </c>
       <c r="D14">
-        <v>0.04395726403373454</v>
+        <v>0.03977016629572373</v>
       </c>
       <c r="E14">
-        <v>0.01294391817101747</v>
+        <v>0.01312045464117798</v>
       </c>
       <c r="F14">
-        <v>3.395978207909147</v>
+        <v>3.031157637701577</v>
       </c>
       <c r="G14">
-        <v>0.0006838380380090882</v>
+        <v>0.002436180226870007</v>
       </c>
       <c r="H14">
-        <v>0.01858765059970674</v>
+        <v>0.0140545477382235</v>
       </c>
       <c r="I14">
-        <v>0.06932687746776234</v>
+        <v>0.06548578485322396</v>
       </c>
     </row>
     <row r="15">
@@ -873,22 +873,22 @@
         </is>
       </c>
       <c r="D15">
-        <v>0.03617319801135294</v>
+        <v>0.03984602158473804</v>
       </c>
       <c r="E15">
-        <v>0.01187941764085821</v>
+        <v>0.01232359588857734</v>
       </c>
       <c r="F15">
-        <v>3.045031255314942</v>
+        <v>3.233311279029448</v>
       </c>
       <c r="G15">
-        <v>0.002326561303417791</v>
+        <v>0.001223641535237426</v>
       </c>
       <c r="H15">
-        <v>0.01288996727796108</v>
+        <v>0.01569221748310058</v>
       </c>
       <c r="I15">
-        <v>0.0594564287447448</v>
+        <v>0.06399982568637549</v>
       </c>
     </row>
     <row r="16">
@@ -908,22 +908,22 @@
         </is>
       </c>
       <c r="D16">
-        <v>0.05122854673723441</v>
+        <v>0.05244259081769893</v>
       </c>
       <c r="E16">
-        <v>7.323335287014129E-05</v>
+        <v>9.226942806137777E-05</v>
       </c>
       <c r="F16">
-        <v>699.5248029688576</v>
+        <v>568.3636706061951</v>
       </c>
       <c r="G16">
         <v>0</v>
       </c>
       <c r="H16">
-        <v>0.05108501200314181</v>
+        <v>0.05226174606182452</v>
       </c>
       <c r="I16">
-        <v>0.051372081471327</v>
+        <v>0.05262343557357334</v>
       </c>
     </row>
     <row r="17">
@@ -943,22 +943,22 @@
         </is>
       </c>
       <c r="D17">
-        <v>0.08721185842610392</v>
+        <v>0.1047352533767841</v>
       </c>
       <c r="E17">
-        <v>0.01848201416762753</v>
+        <v>0.01937877648231309</v>
       </c>
       <c r="F17">
-        <v>4.718742104356854</v>
+        <v>5.404637050867245</v>
       </c>
       <c r="G17">
-        <v>2.373074312260175E-06</v>
+        <v>6.493975409178787E-08</v>
       </c>
       <c r="H17">
-        <v>0.05098777629579494</v>
+        <v>0.06675354940699868</v>
       </c>
       <c r="I17">
-        <v>0.1234359405564129</v>
+        <v>0.1427169573465696</v>
       </c>
     </row>
     <row r="18">
@@ -978,22 +978,22 @@
         </is>
       </c>
       <c r="D18">
-        <v>0.06127645439837474</v>
+        <v>0.05193726163737072</v>
       </c>
       <c r="E18">
-        <v>0.02254362136675461</v>
+        <v>0.02325225627984554</v>
       </c>
       <c r="F18">
-        <v>2.718128263489201</v>
+        <v>2.233643953184389</v>
       </c>
       <c r="G18">
-        <v>0.00656523823248838</v>
+        <v>0.0255065094659875</v>
       </c>
       <c r="H18">
-        <v>0.0170917684384281</v>
+        <v>0.006363676769578164</v>
       </c>
       <c r="I18">
-        <v>0.1054611403583214</v>
+        <v>0.09751084650516328</v>
       </c>
     </row>
     <row r="19">
@@ -1013,22 +1013,22 @@
         </is>
       </c>
       <c r="D19">
-        <v>0.0572620115684157</v>
+        <v>0.06480183153932956</v>
       </c>
       <c r="E19">
-        <v>0.02159849990921959</v>
+        <v>0.02305151583207117</v>
       </c>
       <c r="F19">
-        <v>2.651203176567494</v>
+        <v>2.811174415227475</v>
       </c>
       <c r="G19">
-        <v>0.008020557677239592</v>
+        <v>0.004936102005392109</v>
       </c>
       <c r="H19">
-        <v>0.01492972962625369</v>
+        <v>0.01962169071941523</v>
       </c>
       <c r="I19">
-        <v>0.09959429351057772</v>
+        <v>0.1099819723592439</v>
       </c>
     </row>
     <row r="20">
@@ -1048,22 +1048,22 @@
         </is>
       </c>
       <c r="D20">
-        <v>0.00555198037903053</v>
+        <v>0.0050118114917662</v>
       </c>
       <c r="E20">
-        <v>0.003179220409531464</v>
+        <v>0.003229747794481636</v>
       </c>
       <c r="F20">
-        <v>1.746333900721514</v>
+        <v>1.551765589972507</v>
       </c>
       <c r="G20">
-        <v>0.08075294836846124</v>
+        <v>0.1207183221815232</v>
       </c>
       <c r="H20">
-        <v>-0.0006791771225658199</v>
+        <v>-0.001318377864565477</v>
       </c>
       <c r="I20">
-        <v>0.01178313788062688</v>
+        <v>0.01134200084809788</v>
       </c>
     </row>
     <row r="21">
@@ -1083,22 +1083,22 @@
         </is>
       </c>
       <c r="D21">
-        <v>0.005521536654153434</v>
+        <v>0.004459276853191458</v>
       </c>
       <c r="E21">
-        <v>0.004600410495271725</v>
+        <v>0.004538491916662724</v>
       </c>
       <c r="F21">
-        <v>1.200226949275165</v>
+        <v>0.9825459503011487</v>
       </c>
       <c r="G21">
-        <v>0.2300512116763225</v>
+        <v>0.3258309571033339</v>
       </c>
       <c r="H21">
-        <v>-0.003495102230679216</v>
+        <v>-0.00443600384759364</v>
       </c>
       <c r="I21">
-        <v>0.01453817553898609</v>
+        <v>0.01335455755397656</v>
       </c>
     </row>
     <row r="22">
@@ -1118,22 +1118,22 @@
         </is>
       </c>
       <c r="D22">
-        <v>0.003924398627270106</v>
+        <v>0.001050349619761949</v>
       </c>
       <c r="E22">
-        <v>0.00439050095017047</v>
+        <v>0.004545355113149121</v>
       </c>
       <c r="F22">
-        <v>0.8938384644052368</v>
+        <v>0.2310819712905212</v>
       </c>
       <c r="G22">
-        <v>0.3714083257845591</v>
+        <v>0.8172511209337914</v>
       </c>
       <c r="H22">
-        <v>-0.004680825109152899</v>
+        <v>-0.007858382698955309</v>
       </c>
       <c r="I22">
-        <v>0.01252962236369311</v>
+        <v>0.009959081938479207</v>
       </c>
     </row>
     <row r="23">
@@ -1153,22 +1153,22 @@
         </is>
       </c>
       <c r="D23">
-        <v>0.002002029479148448</v>
+        <v>0.0006825039839203173</v>
       </c>
       <c r="E23">
-        <v>0.003384288249707309</v>
+        <v>4.443660587626631E-05</v>
       </c>
       <c r="F23">
-        <v>0.5915658866592094</v>
+        <v>15.35904847955195</v>
       </c>
       <c r="G23">
-        <v>0.5541413229786467</v>
+        <v>3.080628498892604E-53</v>
       </c>
       <c r="H23">
-        <v>-0.004631053603579974</v>
+        <v>0.0005954098368076344</v>
       </c>
       <c r="I23">
-        <v>0.00863511256187687</v>
+        <v>0.0007695981310330001</v>
       </c>
     </row>
     <row r="24">
@@ -1188,22 +1188,22 @@
         </is>
       </c>
       <c r="D24">
-        <v>-0.009289013825161148</v>
+        <v>0.00336897099845952</v>
       </c>
       <c r="E24">
-        <v>0.003365158115142569</v>
+        <v>0.003916198991833251</v>
       </c>
       <c r="F24">
-        <v>-2.76034988768057</v>
+        <v>0.8602655292759873</v>
       </c>
       <c r="G24">
-        <v>0.005773948609862091</v>
+        <v>0.3896426897889415</v>
       </c>
       <c r="H24">
-        <v>-0.01588460253312327</v>
+        <v>-0.00430663798182572</v>
       </c>
       <c r="I24">
-        <v>-0.002693425117199022</v>
+        <v>0.01104457997874476</v>
       </c>
     </row>
     <row r="25">
@@ -1223,22 +1223,22 @@
         </is>
       </c>
       <c r="D25">
-        <v>-0.0006837393394220906</v>
+        <v>0.001227185205059252</v>
       </c>
       <c r="E25">
-        <v>0.01071535417695656</v>
+        <v>0.01089481814254631</v>
       </c>
       <c r="F25">
-        <v>-0.06380930841207996</v>
+        <v>0.1126393473487055</v>
       </c>
       <c r="G25">
-        <v>0.9491220663248111</v>
+        <v>0.9103164888707682</v>
       </c>
       <c r="H25">
-        <v>-0.02168544760784778</v>
+        <v>-0.02012626597244507</v>
       </c>
       <c r="I25">
-        <v>0.0203179689290036</v>
+        <v>0.02258063638256358</v>
       </c>
     </row>
     <row r="26">
@@ -1258,22 +1258,22 @@
         </is>
       </c>
       <c r="D26">
-        <v>0.01549924898784005</v>
+        <v>0.01915780019998702</v>
       </c>
       <c r="E26">
-        <v>0.009188158282776167</v>
+        <v>0.009506307602736097</v>
       </c>
       <c r="F26">
-        <v>1.686872223010617</v>
+        <v>2.015272490706385</v>
       </c>
       <c r="G26">
-        <v>0.09162792422352779</v>
+        <v>0.04387610566430804</v>
       </c>
       <c r="H26">
-        <v>-0.002509210330654625</v>
+        <v>0.0005257796726649729</v>
       </c>
       <c r="I26">
-        <v>0.03350770830633472</v>
+        <v>0.03778982072730906</v>
       </c>
     </row>
     <row r="27">
@@ -1293,22 +1293,22 @@
         </is>
       </c>
       <c r="D27">
-        <v>0.01482409799661824</v>
+        <v>0.01383760620407962</v>
       </c>
       <c r="E27">
-        <v>0.01633031008714191</v>
+        <v>0.01658081415119263</v>
       </c>
       <c r="F27">
-        <v>0.907765860997972</v>
+        <v>0.8345552925146507</v>
       </c>
       <c r="G27">
-        <v>0.3640019388040006</v>
+        <v>0.4039681431592572</v>
       </c>
       <c r="H27">
-        <v>-0.01718272163055104</v>
+        <v>-0.01866019236660998</v>
       </c>
       <c r="I27">
-        <v>0.04683091762378752</v>
+        <v>0.04633540477476923</v>
       </c>
     </row>
     <row r="28">
@@ -1328,22 +1328,22 @@
         </is>
       </c>
       <c r="D28">
-        <v>-0.0201188620382464</v>
+        <v>-0.02875493208931094</v>
       </c>
       <c r="E28">
-        <v>0.01539912173057227</v>
+        <v>0.01623552039303771</v>
       </c>
       <c r="F28">
-        <v>-1.306494122863118</v>
+        <v>-1.771112437002138</v>
       </c>
       <c r="G28">
-        <v>0.1913845763565469</v>
+        <v>0.07654200624551558</v>
       </c>
       <c r="H28">
-        <v>-0.05030058602371616</v>
+        <v>-0.06057596732993044</v>
       </c>
       <c r="I28">
-        <v>0.01006286194722335</v>
+        <v>0.003066103151308553</v>
       </c>
     </row>
   </sheetData>

</xml_diff>